<commit_message>
2026 water quality data processing, updating AGRRA plots
</commit_message>
<xml_diff>
--- a/agrra_monitoring/data_raw/ATG_NEMMA_2025/Calculated/BenthicAlgalHeight.xlsx
+++ b/agrra_monitoring/data_raw/ATG_NEMMA_2025/Calculated/BenthicAlgalHeight.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\ATG\Calculated\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\AGRRA Group Work\Data Product Fix\Ruleo\NEMMA&amp;CadesReef2025\Calculated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695F3893-EDC5-474B-A464-6699D8A7F52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F1D491D-8024-4BE1-8F04-F9E8F245DB0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-45" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="TermsOfUse" sheetId="4" r:id="rId1"/>
+    <sheet name="TermsOfUse" sheetId="5" r:id="rId1"/>
     <sheet name="Metadata" sheetId="1" r:id="rId2"/>
     <sheet name="Standard" sheetId="2" r:id="rId3"/>
     <sheet name="Scaled" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="999999"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -340,48 +340,39 @@
     <t>tFMA-P</t>
   </si>
   <si>
-    <t>Created: 2025 May 29</t>
-  </si>
-  <si>
-    <t>Version 1.0</t>
-  </si>
-  <si>
+    <t>Created: 2026 May 29</t>
+  </si>
+  <si>
+    <t>AGRRA Terms of Data Service</t>
+  </si>
+  <si>
+    <t>The Atlantic and Gulf Rapid Reef Assessment (AGRRA) Program champions coral reef conservation and empowers those who protect these diverse ecosystems. We are an international collaboration of scientists, managers, and supporters aimed at improving the regional condition of reefs in the Western Atlantic and Gulf of Mexico. For 25 years, AGRRA has used an innovative regional approach to examine the condition of reef-building corals, algae, and fishes, and support the conservation of coral reef ecosystems. We curate and distribute data, research and educational materials that support this mission. For more information, visit www.agrra.org or email info@agrra.org.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">AGRRA’s goal is to provide data contributors access to the AGRRA data platform, which provides: 
+a)	a standardized way to enter coral reef monitoring data with built in quality controls,
+b)	an efficient way to process data and visualize data through interactive graphics,
+c)	synthesized data products provided as RAW data and Calculated Products, and 
+d)	a centralized and secure place to manage and store data.
+</t>
+    </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="13"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Date produced: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">Data in this country batch were produced in collaboration with the batch owner: Margaret Wilson. These data products are in draft form and are under review. Prior to data use, you need to accept the Terms and Conditions in the AGRRA Data License below. In addition, permission to distribute data must follow any data agreements required by the batch owner and/or individual surveyors who submitted data prior to use. </t>
-    </r>
-  </si>
-  <si>
-    <t>The Atlantic and Gulf Rapid Reef Assessment (AGRRA) Program champions coral reef conservation and empowers those who protect these diverse ecosystems. We are an international collaboration of scientists, managers, and supporters aimed at improving the regional condition of reefs in the Western Atlantic and Gulf of Mexico. For 25 years, AGRRA has used an innovative regional approach to examine the condition of reef-building corals, algae and fishes and support the conservation of coral reef ecosystems. We curate and distribute data, research and educational materials that support this mission. For more information, visit www.agrra.org or email info@agrra.org.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Conditions of Use of AGRRA Data Products
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">In order to use the AGRRA dataset, you need to accept the Terms and Conditions in the AGRRA Data License below.
-</t>
+      <t xml:space="preserve">
+1. Ownership &amp; Intellectual Property</t>
     </r>
     <r>
       <rPr>
@@ -392,7 +383,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>AGRRA Data License and Data Use Agreements</t>
+      <t xml:space="preserve">
+</t>
     </r>
     <r>
       <rPr>
@@ -400,9 +392,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">
-By accessing and using any of the datasets distributed by AGRRA, you acknowledge that you have read, understood, and agree to comply with the terms and conditions contained within this agreement. A Data Use Agreement (DUA) must be entered into before there is any use or distribution of a data set to an outside entity. AGRRA may amend these terms and conditions at any time. Your continued use of this data constitutes acceptance of the terms and conditions stated at the time of your use. You should contact AGRRA to determine the current terms and conditions to which you are bound.
-</t>
+      <t xml:space="preserve">•	</t>
     </r>
     <r>
       <rPr>
@@ -413,7 +403,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Data Permissions and Proprietary Rights to Content</t>
+      <t>Original Observations:</t>
     </r>
     <r>
       <rPr>
@@ -421,9 +411,8 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">
-All datasets are the property of AGRRA and/or its affiliates, unless otherwise noted. With permission and DUA, you may use these datasets for non-commercial purposes, including research, education, presentations, and non-commercial publications. You understand and agree that you may not copy, reproduce, distribute or create derivative works for other purposes, without prior, written authorization from the AGRRA Project Leader. When using or publishing any parts of these datasets, proper acknowledgement of AGRRA and original source(s), is required.
-</t>
+      <t xml:space="preserve"> The raw data collected during surveys remains the intellectual property of the original data collectors and their respective organizations.
+•	</t>
     </r>
     <r>
       <rPr>
@@ -434,7 +423,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Limitation of Liability</t>
+      <t xml:space="preserve">Methodology &amp; Systems: </t>
     </r>
     <r>
       <rPr>
@@ -442,9 +431,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">
-AGRRA makes reasonable efforts to provide accurate data and information through its website, database, and other channels. Nevertheless, you understand and agree that AGRRA shall not be liable for any loss or damage resulting from any use of, or inability to use, this data, or resulting from any errors or omissions in the data content.
-</t>
+      <t xml:space="preserve">All protocols (Benthic, Coral, Fish), platform systems, AGRRA content, and related tools remain the intellectual property of </t>
     </r>
     <r>
       <rPr>
@@ -455,7 +442,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Data Citation </t>
+      <t>Ocean Research &amp; Education Foundation, Inc. (ORE)</t>
     </r>
     <r>
       <rPr>
@@ -463,9 +450,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">
-For any use of AGRRA data or datasets managed by AGRRA, or for general reference to the project in peer-reviewed literature, use the citation specified in the data use policy or for general citation use the following format below to cite data retrieved from the AGRRA website or AGRRA database manager. 
-</t>
+      <t xml:space="preserve">, </t>
     </r>
     <r>
       <rPr>
@@ -476,7 +461,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Citation:</t>
+      <t>AGRRA</t>
     </r>
     <r>
       <rPr>
@@ -484,8 +469,8 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve"> AGRRA. 2024. Atlantic and Gulf Rapid Reef Assessment (AGRRA): An online database of AGRRA coral reef survey data. Available: http://agrra.org. (Accessed: Date [e.g., March 10, 2024]).
-</t>
+      <t xml:space="preserve">, and their licensors, as applicable.
+•	</t>
     </r>
     <r>
       <rPr>
@@ -496,7 +481,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Acknowledgement:</t>
+      <t xml:space="preserve">Processed Metrics: </t>
     </r>
     <r>
       <rPr>
@@ -504,11 +489,8 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve"> For general data, use: “We thank the following data providers: Atlantic Gulf Rapid Reef Assessment (AGRRA) contributors and data managers…”. Where noted, individual data contributors should be included in acknowledgments. 
-</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">The calculated metrics, custom-coded logic, and standardized protocols used to generate these spreadsheets are the proprietary property of </t>
+    </r>
     <r>
       <rPr>
         <b/>
@@ -518,7 +500,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Data Use Policy</t>
+      <t>AGRRA</t>
     </r>
     <r>
       <rPr>
@@ -526,19 +508,8 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">
-Data collected under the auspices of AGRRA are available to the public after primary publication, or at most two years after the completion of the study unless proprietary restrictions are warranted. Request for the use of AGRRA data is to be made in writing and is subject to acceptance of the following conditions:
-1. The user agrees to provide valid name and contact information prior to requesting or downloading online data. This information will be used to ensure data agreements are in place, to contact the user in case of changes to the data, and may also be used by data set authors and AGRRA project administrators to document data usage.
-2. The user agrees to cite the data set author (if stated) and AGRRA in all publications in which the data are used, as per the instructions in “Data Citation”. 
-3. The user agrees to provide one copy of any manuscript based on AGRRA data to the AGRRA or data set author (if specified) prior to submitting it for peer-reviewed publication.
-4. The user also agrees to send one electronic copy or reports or publication (pdf format) to: data@agrra.org and gis@agrra.org. 
-5. Users are prohibited from selling or redistributing any data provided by AGRRA without explicit prior permission.
-6. If specified, users are to contact original investigators or data contributors responsible for data prior to data use, and where appropriate, are encouraged to consider collaboration and/or co-authorship with original investigators.
-7. Extensive efforts are made to ensure that data products are accurate and up to date, but the authors and AGRRA will not take responsibility for any errors that may exist in data provided. The user assumes all responsibility for errors in analysis or judgment resulting from use of the data.
-8. Any violation of the terms of this agreement will result in immediate forfeiture of the data and loss of access privileges to other AGRRA data sets.  </t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve"> and the </t>
+    </r>
     <r>
       <rPr>
         <b/>
@@ -548,7 +519,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Format of Data:</t>
+      <t>Ocean Research &amp; Education Foundation (ORE)</t>
     </r>
     <r>
       <rPr>
@@ -556,10 +527,9 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve"> Original data is submitted into the data portal by surveyors trained in the AGRRA method to maintain data accuracy and consistency. AGRRA provides data products as raw products and as calculated products. Note these are draft data products from the beta version of the new AGRRA data portal (2024) and are currently in review. AGRRA reserves the right to update data products as needed.  Contact AGRRA if you have questions.</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">.
+•	</t>
+    </r>
     <r>
       <rPr>
         <b/>
@@ -569,6 +539,601 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t xml:space="preserve">User Content: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Users retain ownership of data, images, and other content they submit, but grant AGRRA the rights needed to store, process, share, and display that content in accordance with these terms.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+2. Data Sharing &amp; Privacy Publication Protocol
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">AGRRA is committed to protecting the privacy of the Data Contributors with respect to their data batches and offers three privacy options for each data batch:
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Batch Privacy Options: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Data Batches may be designated as Private, Public Summary, or Public. Some batch metadata may remain publicly visible to support transparency and attribution.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Accounts &amp; Security:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Data Contributors are responsible for their accounts, passwords, and all activity under their accounts, and must promptly report any suspected unauthorized access.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+3. Permitted Uses</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+•	Non-Commercial Use:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Data Contributors and Third-party Users (with permission) are licensed to use these materials and datasets for research, education, conservation, and other non-commercial purposes.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Commercial Use:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Commercial use, sale, or redistribution of AGRRA materials, datasets, or API outputs requires prior written permission.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lawful and Responsible Use:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> All users must comply with applicable laws and must not misuse, disrupt, alter, scrape, or interfere with the platform, its software, security, or other users.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+4. Citation &amp; Acknowledgment
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A. Guidance for Original Data Contributors</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>How to cite your data:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> When publishing, presenting, or otherwise sharing analyses based on your own contributed dataset, please cite the dataset using the suggested AGRRA format: [Surveyor Names/Organization], [Country] ([Year]). [Dataset Name/Region]. In: Atlantic and Gulf Rapid Reef Assessment (AGRRA) Program Data Platform, [Protocol Version Number] [Data Product Name]. [URL/DOI]. Accessed [Date].
+                o   Examples
+                         ▪For a specific survey: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Smith, J. &amp; Reef Care Bahamas, Bahamas (2024). New Providence Benthic Surveys. In: Atlantic and Gulf Rapid Reef Assessment (AGRRA) Program Data Platform, v5.2 Coral &amp; Benthic Data. www.agrra.org. Accessed May 14, 2026.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+                         ▪For an aggregated country-level report: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Belize Fisheries Department &amp; Healthy Reefs Initiative, Belize (2025). 2025 National Monitoring Data. In: Atlantic and Gulf Rapid Reef Assessment (AGRRA) Program Data Platform. www.agrra.org. Accessed May 2026.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>How to acknowledge AGRRA:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> In all publications and presentations using your contributed data, please acknowledge AGRRA as the platform that curates, manages, and provides access to the dataset.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Suggested acknowledgment language:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "We acknowledge (or thank) the Atlantic and Gulf Rapid Reef Assessment (AGRRA) Program Data Platform for curating and providing access to the dataset used in this work."
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Collaboration:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Contributors are encouraged to remain available for collaboration when their expertise may strengthen data interpretation or publication.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Notification of use:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Please share an electronic copy of any final reports, publications, or presentations with AGRRA curated data to data@agrra.org.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>B. Guidance for Third-Party Data Users</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+Third-party users (not original data collectors) who would like to use an AGRRA data batch should first contact and obtain permission from the original data contributor and/or AGRRA at data@agrra.org. Once permission is granted, third-party users who utilize AGRRA-hosted data for research, presentations, reports, or publications shall give appropriate credit to both the original data contributors and AGRRA. The guidance below explains how to cite the original dataset and how to acknowledge AGRRA as the data platform.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">How to cite original data contributors: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Cite the dataset using the names of the original surveyors, organizations, country, year, and dataset title, following the AGRRA dataset citation format. AGRRA can provide guidance on the appropriate citation for the specific dataset used.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>How to acknowledge AGRRA:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> In addition to citing the original dataset, acknowledge the Atlantic and Gulf Rapid Reef Assessment (AGRRA) Program Data Platform as the system that curates, manages, and provides access to the data.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Suggested acknowledgment language: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"We thank the original data contributors [insert surveyor and/or organization names, where available] and acknowledge the Atlantic and Gulf Rapid Reef Assessment (AGRRA) Program Data Platform for curating and providing access to the dataset used in this work."
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Direct contact and collaboration:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Third-party users are encouraged to contact the original data collectors to discuss collaboration or co-authorship, clarify interpretation, and share findings, where appropriate.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+5. Liability &amp; Compliance
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Integrity:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> AGRRA works diligently to maintain data accuracy; however, Data Contributors and Third-Party users are responsible for their own analyses, interpretations, and resulting conclusions.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No Warranty:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> The platform, data, and related content are provided “as is” and “as available,” without guarantees of accuracy, availability, security, or fitness for a particular purpose.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Limitation of Liability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> AGRRA and its operators are not liable for indirect, incidental, consequential, or data-loss-related damages arising from the use of the platform.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Access Review: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">If these terms are not followed, AGRRA reserves the right to review, suspend, modify, or terminate access privileges or service availability as appropriate.
+•	</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Changes &amp; Governing Law:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> AGRRA may update these terms from time to time; continued use represents acceptance. </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">           </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Metadata:</t>
     </r>
     <r>
@@ -581,23 +1146,30 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
+    <t>Version 1.0</t>
+  </si>
+  <si>
+    <t>Data provided in these country batches were produced in collaboration with the batch owner: Ruleo Camacho. Prior to data use, you need to accept the Terms and Conditions in the AGRRA Terms of Data Service below. In addition, permission to distribute data must follow any data agreements required by the batch owner and/or individual surveyors who submitted data prior to use.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
-      </rPr>
-      <t>©</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Ocean Research and Education Foundation</t>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Format of Data:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Original data is submitted into the data portal by surveyors trained in the AGRRA method to maintain data accuracy and consistency. AGRRA provides data products as raw products and as calculated products. AGRRA reserves the right to update data products as needed.  Contact AGRRA if you have questions.</t>
     </r>
   </si>
 </sst>
@@ -608,11 +1180,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0#"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -636,16 +1215,35 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -668,7 +1266,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -686,6 +1284,66 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -695,7 +1353,22 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -818,16 +1491,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -853,126 +1527,117 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{9329BBCB-D3D6-4CB2-A29A-3873149B48FA}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{D8BDAEE4-47C6-4CB9-9FE8-0B4CB12A5199}"/>
+    <cellStyle name="Normal 2 2" xfId="2" xr:uid="{7EB11FA0-E592-4237-B5AF-90D4AB2E6C07}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
@@ -985,61 +1650,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>257176</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>180976</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>322132</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>123826</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{458885D6-7C15-4F87-91CF-A88DDCFA0195}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6276976" y="180976"/>
-          <a:ext cx="2655756" cy="2038350"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1328,1057 +1938,1607 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CEBBB7D-D923-4D9D-9BDE-E8697D8E2108}">
-  <dimension ref="A1:W78"/>
-  <sheetFormatPr defaultColWidth="9.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D2F5C1-7FA9-4287-8B61-2018EF143BA3}">
+  <dimension ref="A1:X70"/>
+  <sheetFormatPr defaultColWidth="9.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" style="17" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" style="17" customWidth="1"/>
-    <col min="3" max="16384" width="9.7109375" style="17"/>
+    <col min="2" max="2" width="11.26953125" style="17" customWidth="1"/>
+    <col min="3" max="16384" width="9.7265625" style="17"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>105</v>
       </c>
       <c r="B1" s="16"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="16"/>
+    </row>
+    <row r="4" spans="1:23" ht="19.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="16"/>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+    </row>
+    <row r="5" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A6" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="22"/>
+    </row>
+    <row r="7" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="23"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="24"/>
+      <c r="Q7" s="24"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24"/>
+      <c r="T7" s="24"/>
+      <c r="U7" s="24"/>
+      <c r="V7" s="24"/>
+      <c r="W7" s="25"/>
+    </row>
+    <row r="8" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="9" spans="1:23" ht="53.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
-      <c r="M13" s="18"/>
-      <c r="N13" s="18"/>
-      <c r="O13" s="18"/>
-      <c r="P13" s="18"/>
-      <c r="Q13" s="18"/>
-      <c r="R13" s="18"/>
-      <c r="S13" s="18"/>
-      <c r="T13" s="18"/>
-      <c r="U13" s="18"/>
-      <c r="V13" s="18"/>
-      <c r="W13" s="18"/>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A14" s="18"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="18"/>
-      <c r="P14" s="18"/>
-      <c r="Q14" s="18"/>
-      <c r="R14" s="18"/>
-      <c r="S14" s="18"/>
-      <c r="T14" s="18"/>
-      <c r="U14" s="18"/>
-      <c r="V14" s="18"/>
-      <c r="W14" s="18"/>
-    </row>
-    <row r="15" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:23" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="19" t="s">
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="27"/>
+      <c r="M9" s="27"/>
+      <c r="N9" s="27"/>
+      <c r="O9" s="27"/>
+      <c r="P9" s="27"/>
+      <c r="Q9" s="27"/>
+      <c r="R9" s="27"/>
+      <c r="S9" s="27"/>
+      <c r="T9" s="27"/>
+      <c r="U9" s="27"/>
+      <c r="V9" s="27"/>
+      <c r="W9" s="28"/>
+    </row>
+    <row r="10" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="20"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="20"/>
-      <c r="Q16" s="20"/>
-      <c r="R16" s="20"/>
-      <c r="S16" s="20"/>
-      <c r="T16" s="20"/>
-      <c r="U16" s="20"/>
-      <c r="V16" s="20"/>
-      <c r="W16" s="21"/>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="30"/>
+      <c r="P10" s="30"/>
+      <c r="Q10" s="30"/>
+      <c r="R10" s="30"/>
+      <c r="S10" s="30"/>
+      <c r="T10" s="30"/>
+      <c r="U10" s="30"/>
+      <c r="V10" s="30"/>
+      <c r="W10" s="31"/>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A11" s="32"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="33"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="33"/>
+      <c r="L11" s="33"/>
+      <c r="M11" s="33"/>
+      <c r="N11" s="33"/>
+      <c r="O11" s="33"/>
+      <c r="P11" s="33"/>
+      <c r="Q11" s="33"/>
+      <c r="R11" s="33"/>
+      <c r="S11" s="33"/>
+      <c r="T11" s="33"/>
+      <c r="U11" s="33"/>
+      <c r="V11" s="33"/>
+      <c r="W11" s="34"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A12" s="32"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="33"/>
+      <c r="M12" s="33"/>
+      <c r="N12" s="33"/>
+      <c r="O12" s="33"/>
+      <c r="P12" s="33"/>
+      <c r="Q12" s="33"/>
+      <c r="R12" s="33"/>
+      <c r="S12" s="33"/>
+      <c r="T12" s="33"/>
+      <c r="U12" s="33"/>
+      <c r="V12" s="33"/>
+      <c r="W12" s="34"/>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A13" s="32"/>
+      <c r="B13" s="33"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="33"/>
+      <c r="J13" s="33"/>
+      <c r="K13" s="33"/>
+      <c r="L13" s="33"/>
+      <c r="M13" s="33"/>
+      <c r="N13" s="33"/>
+      <c r="O13" s="33"/>
+      <c r="P13" s="33"/>
+      <c r="Q13" s="33"/>
+      <c r="R13" s="33"/>
+      <c r="S13" s="33"/>
+      <c r="T13" s="33"/>
+      <c r="U13" s="33"/>
+      <c r="V13" s="33"/>
+      <c r="W13" s="34"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A14" s="32"/>
+      <c r="B14" s="33"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="33"/>
+      <c r="J14" s="33"/>
+      <c r="K14" s="33"/>
+      <c r="L14" s="33"/>
+      <c r="M14" s="33"/>
+      <c r="N14" s="33"/>
+      <c r="O14" s="33"/>
+      <c r="P14" s="33"/>
+      <c r="Q14" s="33"/>
+      <c r="R14" s="33"/>
+      <c r="S14" s="33"/>
+      <c r="T14" s="33"/>
+      <c r="U14" s="33"/>
+      <c r="V14" s="33"/>
+      <c r="W14" s="34"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A15" s="32"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+      <c r="J15" s="33"/>
+      <c r="K15" s="33"/>
+      <c r="L15" s="33"/>
+      <c r="M15" s="33"/>
+      <c r="N15" s="33"/>
+      <c r="O15" s="33"/>
+      <c r="P15" s="33"/>
+      <c r="Q15" s="33"/>
+      <c r="R15" s="33"/>
+      <c r="S15" s="33"/>
+      <c r="T15" s="33"/>
+      <c r="U15" s="33"/>
+      <c r="V15" s="33"/>
+      <c r="W15" s="34"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A16" s="32"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+      <c r="P16" s="33"/>
+      <c r="Q16" s="33"/>
+      <c r="R16" s="33"/>
+      <c r="S16" s="33"/>
+      <c r="T16" s="33"/>
+      <c r="U16" s="33"/>
+      <c r="V16" s="33"/>
+      <c r="W16" s="34"/>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A17" s="32"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="33"/>
+      <c r="K17" s="33"/>
+      <c r="L17" s="33"/>
+      <c r="M17" s="33"/>
+      <c r="N17" s="33"/>
+      <c r="O17" s="33"/>
+      <c r="P17" s="33"/>
+      <c r="Q17" s="33"/>
+      <c r="R17" s="33"/>
+      <c r="S17" s="33"/>
+      <c r="T17" s="33"/>
+      <c r="U17" s="33"/>
+      <c r="V17" s="33"/>
+      <c r="W17" s="34"/>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A18" s="32"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="33"/>
+      <c r="K18" s="33"/>
+      <c r="L18" s="33"/>
+      <c r="M18" s="33"/>
+      <c r="N18" s="33"/>
+      <c r="O18" s="33"/>
+      <c r="P18" s="33"/>
+      <c r="Q18" s="33"/>
+      <c r="R18" s="33"/>
+      <c r="S18" s="33"/>
+      <c r="T18" s="33"/>
+      <c r="U18" s="33"/>
+      <c r="V18" s="33"/>
+      <c r="W18" s="34"/>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A19" s="32"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="33"/>
+      <c r="M19" s="33"/>
+      <c r="N19" s="33"/>
+      <c r="O19" s="33"/>
+      <c r="P19" s="33"/>
+      <c r="Q19" s="33"/>
+      <c r="R19" s="33"/>
+      <c r="S19" s="33"/>
+      <c r="T19" s="33"/>
+      <c r="U19" s="33"/>
+      <c r="V19" s="33"/>
+      <c r="W19" s="34"/>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A20" s="32"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="33"/>
+      <c r="N20" s="33"/>
+      <c r="O20" s="33"/>
+      <c r="P20" s="33"/>
+      <c r="Q20" s="33"/>
+      <c r="R20" s="33"/>
+      <c r="S20" s="33"/>
+      <c r="T20" s="33"/>
+      <c r="U20" s="33"/>
+      <c r="V20" s="33"/>
+      <c r="W20" s="34"/>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A21" s="32"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
+      <c r="J21" s="33"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="33"/>
+      <c r="N21" s="33"/>
+      <c r="O21" s="33"/>
+      <c r="P21" s="33"/>
+      <c r="Q21" s="33"/>
+      <c r="R21" s="33"/>
+      <c r="S21" s="33"/>
+      <c r="T21" s="33"/>
+      <c r="U21" s="33"/>
+      <c r="V21" s="33"/>
+      <c r="W21" s="34"/>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A22" s="32"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+      <c r="N22" s="33"/>
+      <c r="O22" s="33"/>
+      <c r="P22" s="33"/>
+      <c r="Q22" s="33"/>
+      <c r="R22" s="33"/>
+      <c r="S22" s="33"/>
+      <c r="T22" s="33"/>
+      <c r="U22" s="33"/>
+      <c r="V22" s="33"/>
+      <c r="W22" s="34"/>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A23" s="32"/>
+      <c r="B23" s="33"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="33"/>
+      <c r="J23" s="33"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="33"/>
+      <c r="N23" s="33"/>
+      <c r="O23" s="33"/>
+      <c r="P23" s="33"/>
+      <c r="Q23" s="33"/>
+      <c r="R23" s="33"/>
+      <c r="S23" s="33"/>
+      <c r="T23" s="33"/>
+      <c r="U23" s="33"/>
+      <c r="V23" s="33"/>
+      <c r="W23" s="34"/>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A24" s="32"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+      <c r="J24" s="33"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="33"/>
+      <c r="N24" s="33"/>
+      <c r="O24" s="33"/>
+      <c r="P24" s="33"/>
+      <c r="Q24" s="33"/>
+      <c r="R24" s="33"/>
+      <c r="S24" s="33"/>
+      <c r="T24" s="33"/>
+      <c r="U24" s="33"/>
+      <c r="V24" s="33"/>
+      <c r="W24" s="34"/>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A25" s="32"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="33"/>
+      <c r="J25" s="33"/>
+      <c r="K25" s="33"/>
+      <c r="L25" s="33"/>
+      <c r="M25" s="33"/>
+      <c r="N25" s="33"/>
+      <c r="O25" s="33"/>
+      <c r="P25" s="33"/>
+      <c r="Q25" s="33"/>
+      <c r="R25" s="33"/>
+      <c r="S25" s="33"/>
+      <c r="T25" s="33"/>
+      <c r="U25" s="33"/>
+      <c r="V25" s="33"/>
+      <c r="W25" s="34"/>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A26" s="32"/>
+      <c r="B26" s="33"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="33"/>
+      <c r="J26" s="33"/>
+      <c r="K26" s="33"/>
+      <c r="L26" s="33"/>
+      <c r="M26" s="33"/>
+      <c r="N26" s="33"/>
+      <c r="O26" s="33"/>
+      <c r="P26" s="33"/>
+      <c r="Q26" s="33"/>
+      <c r="R26" s="33"/>
+      <c r="S26" s="33"/>
+      <c r="T26" s="33"/>
+      <c r="U26" s="33"/>
+      <c r="V26" s="33"/>
+      <c r="W26" s="34"/>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A27" s="32"/>
+      <c r="B27" s="33"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="33"/>
+      <c r="J27" s="33"/>
+      <c r="K27" s="33"/>
+      <c r="L27" s="33"/>
+      <c r="M27" s="33"/>
+      <c r="N27" s="33"/>
+      <c r="O27" s="33"/>
+      <c r="P27" s="33"/>
+      <c r="Q27" s="33"/>
+      <c r="R27" s="33"/>
+      <c r="S27" s="33"/>
+      <c r="T27" s="33"/>
+      <c r="U27" s="33"/>
+      <c r="V27" s="33"/>
+      <c r="W27" s="34"/>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A28" s="32"/>
+      <c r="B28" s="33"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
+      <c r="K28" s="33"/>
+      <c r="L28" s="33"/>
+      <c r="M28" s="33"/>
+      <c r="N28" s="33"/>
+      <c r="O28" s="33"/>
+      <c r="P28" s="33"/>
+      <c r="Q28" s="33"/>
+      <c r="R28" s="33"/>
+      <c r="S28" s="33"/>
+      <c r="T28" s="33"/>
+      <c r="U28" s="33"/>
+      <c r="V28" s="33"/>
+      <c r="W28" s="34"/>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A29" s="32"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
+      <c r="K29" s="33"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="33"/>
+      <c r="N29" s="33"/>
+      <c r="O29" s="33"/>
+      <c r="P29" s="33"/>
+      <c r="Q29" s="33"/>
+      <c r="R29" s="33"/>
+      <c r="S29" s="33"/>
+      <c r="T29" s="33"/>
+      <c r="U29" s="33"/>
+      <c r="V29" s="33"/>
+      <c r="W29" s="34"/>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A30" s="32"/>
+      <c r="B30" s="33"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="33"/>
+      <c r="N30" s="33"/>
+      <c r="O30" s="33"/>
+      <c r="P30" s="33"/>
+      <c r="Q30" s="33"/>
+      <c r="R30" s="33"/>
+      <c r="S30" s="33"/>
+      <c r="T30" s="33"/>
+      <c r="U30" s="33"/>
+      <c r="V30" s="33"/>
+      <c r="W30" s="34"/>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A31" s="32"/>
+      <c r="B31" s="33"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="33"/>
+      <c r="J31" s="33"/>
+      <c r="K31" s="33"/>
+      <c r="L31" s="33"/>
+      <c r="M31" s="33"/>
+      <c r="N31" s="33"/>
+      <c r="O31" s="33"/>
+      <c r="P31" s="33"/>
+      <c r="Q31" s="33"/>
+      <c r="R31" s="33"/>
+      <c r="S31" s="33"/>
+      <c r="T31" s="33"/>
+      <c r="U31" s="33"/>
+      <c r="V31" s="33"/>
+      <c r="W31" s="34"/>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A32" s="32"/>
+      <c r="B32" s="33"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="33"/>
+      <c r="J32" s="33"/>
+      <c r="K32" s="33"/>
+      <c r="L32" s="33"/>
+      <c r="M32" s="33"/>
+      <c r="N32" s="33"/>
+      <c r="O32" s="33"/>
+      <c r="P32" s="33"/>
+      <c r="Q32" s="33"/>
+      <c r="R32" s="33"/>
+      <c r="S32" s="33"/>
+      <c r="T32" s="33"/>
+      <c r="U32" s="33"/>
+      <c r="V32" s="33"/>
+      <c r="W32" s="34"/>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A33" s="32"/>
+      <c r="B33" s="33"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+      <c r="G33" s="33"/>
+      <c r="H33" s="33"/>
+      <c r="I33" s="33"/>
+      <c r="J33" s="33"/>
+      <c r="K33" s="33"/>
+      <c r="L33" s="33"/>
+      <c r="M33" s="33"/>
+      <c r="N33" s="33"/>
+      <c r="O33" s="33"/>
+      <c r="P33" s="33"/>
+      <c r="Q33" s="33"/>
+      <c r="R33" s="33"/>
+      <c r="S33" s="33"/>
+      <c r="T33" s="33"/>
+      <c r="U33" s="33"/>
+      <c r="V33" s="33"/>
+      <c r="W33" s="34"/>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A34" s="32"/>
+      <c r="B34" s="33"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="33"/>
+      <c r="E34" s="33"/>
+      <c r="F34" s="33"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="33"/>
+      <c r="I34" s="33"/>
+      <c r="J34" s="33"/>
+      <c r="K34" s="33"/>
+      <c r="L34" s="33"/>
+      <c r="M34" s="33"/>
+      <c r="N34" s="33"/>
+      <c r="O34" s="33"/>
+      <c r="P34" s="33"/>
+      <c r="Q34" s="33"/>
+      <c r="R34" s="33"/>
+      <c r="S34" s="33"/>
+      <c r="T34" s="33"/>
+      <c r="U34" s="33"/>
+      <c r="V34" s="33"/>
+      <c r="W34" s="34"/>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A35" s="32"/>
+      <c r="B35" s="33"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="33"/>
+      <c r="E35" s="33"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="33"/>
+      <c r="J35" s="33"/>
+      <c r="K35" s="33"/>
+      <c r="L35" s="33"/>
+      <c r="M35" s="33"/>
+      <c r="N35" s="33"/>
+      <c r="O35" s="33"/>
+      <c r="P35" s="33"/>
+      <c r="Q35" s="33"/>
+      <c r="R35" s="33"/>
+      <c r="S35" s="33"/>
+      <c r="T35" s="33"/>
+      <c r="U35" s="33"/>
+      <c r="V35" s="33"/>
+      <c r="W35" s="34"/>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A36" s="32"/>
+      <c r="B36" s="33"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="33"/>
+      <c r="I36" s="33"/>
+      <c r="J36" s="33"/>
+      <c r="K36" s="33"/>
+      <c r="L36" s="33"/>
+      <c r="M36" s="33"/>
+      <c r="N36" s="33"/>
+      <c r="O36" s="33"/>
+      <c r="P36" s="33"/>
+      <c r="Q36" s="33"/>
+      <c r="R36" s="33"/>
+      <c r="S36" s="33"/>
+      <c r="T36" s="33"/>
+      <c r="U36" s="33"/>
+      <c r="V36" s="33"/>
+      <c r="W36" s="34"/>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A37" s="32"/>
+      <c r="B37" s="33"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="33"/>
+      <c r="E37" s="33"/>
+      <c r="F37" s="33"/>
+      <c r="G37" s="33"/>
+      <c r="H37" s="33"/>
+      <c r="I37" s="33"/>
+      <c r="J37" s="33"/>
+      <c r="K37" s="33"/>
+      <c r="L37" s="33"/>
+      <c r="M37" s="33"/>
+      <c r="N37" s="33"/>
+      <c r="O37" s="33"/>
+      <c r="P37" s="33"/>
+      <c r="Q37" s="33"/>
+      <c r="R37" s="33"/>
+      <c r="S37" s="33"/>
+      <c r="T37" s="33"/>
+      <c r="U37" s="33"/>
+      <c r="V37" s="33"/>
+      <c r="W37" s="34"/>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A38" s="32"/>
+      <c r="B38" s="33"/>
+      <c r="C38" s="33"/>
+      <c r="D38" s="33"/>
+      <c r="E38" s="33"/>
+      <c r="F38" s="33"/>
+      <c r="G38" s="33"/>
+      <c r="H38" s="33"/>
+      <c r="I38" s="33"/>
+      <c r="J38" s="33"/>
+      <c r="K38" s="33"/>
+      <c r="L38" s="33"/>
+      <c r="M38" s="33"/>
+      <c r="N38" s="33"/>
+      <c r="O38" s="33"/>
+      <c r="P38" s="33"/>
+      <c r="Q38" s="33"/>
+      <c r="R38" s="33"/>
+      <c r="S38" s="33"/>
+      <c r="T38" s="33"/>
+      <c r="U38" s="33"/>
+      <c r="V38" s="33"/>
+      <c r="W38" s="34"/>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A39" s="32"/>
+      <c r="B39" s="33"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="33"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="33"/>
+      <c r="J39" s="33"/>
+      <c r="K39" s="33"/>
+      <c r="L39" s="33"/>
+      <c r="M39" s="33"/>
+      <c r="N39" s="33"/>
+      <c r="O39" s="33"/>
+      <c r="P39" s="33"/>
+      <c r="Q39" s="33"/>
+      <c r="R39" s="33"/>
+      <c r="S39" s="33"/>
+      <c r="T39" s="33"/>
+      <c r="U39" s="33"/>
+      <c r="V39" s="33"/>
+      <c r="W39" s="34"/>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A40" s="32"/>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
+      <c r="H40" s="33"/>
+      <c r="I40" s="33"/>
+      <c r="J40" s="33"/>
+      <c r="K40" s="33"/>
+      <c r="L40" s="33"/>
+      <c r="M40" s="33"/>
+      <c r="N40" s="33"/>
+      <c r="O40" s="33"/>
+      <c r="P40" s="33"/>
+      <c r="Q40" s="33"/>
+      <c r="R40" s="33"/>
+      <c r="S40" s="33"/>
+      <c r="T40" s="33"/>
+      <c r="U40" s="33"/>
+      <c r="V40" s="33"/>
+      <c r="W40" s="34"/>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A41" s="32"/>
+      <c r="B41" s="33"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="33"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="33"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="33"/>
+      <c r="K41" s="33"/>
+      <c r="L41" s="33"/>
+      <c r="M41" s="33"/>
+      <c r="N41" s="33"/>
+      <c r="O41" s="33"/>
+      <c r="P41" s="33"/>
+      <c r="Q41" s="33"/>
+      <c r="R41" s="33"/>
+      <c r="S41" s="33"/>
+      <c r="T41" s="33"/>
+      <c r="U41" s="33"/>
+      <c r="V41" s="33"/>
+      <c r="W41" s="34"/>
+      <c r="X41" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="24"/>
-      <c r="L17" s="25" t="s">
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A42" s="32"/>
+      <c r="B42" s="33"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="33"/>
+      <c r="K42" s="33"/>
+      <c r="L42" s="33"/>
+      <c r="M42" s="33"/>
+      <c r="N42" s="33"/>
+      <c r="O42" s="33"/>
+      <c r="P42" s="33"/>
+      <c r="Q42" s="33"/>
+      <c r="R42" s="33"/>
+      <c r="S42" s="33"/>
+      <c r="T42" s="33"/>
+      <c r="U42" s="33"/>
+      <c r="V42" s="33"/>
+      <c r="W42" s="34"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A43" s="32"/>
+      <c r="B43" s="33"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="33"/>
+      <c r="E43" s="33"/>
+      <c r="F43" s="33"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="33"/>
+      <c r="I43" s="33"/>
+      <c r="J43" s="33"/>
+      <c r="K43" s="33"/>
+      <c r="L43" s="33"/>
+      <c r="M43" s="33"/>
+      <c r="N43" s="33"/>
+      <c r="O43" s="33"/>
+      <c r="P43" s="33"/>
+      <c r="Q43" s="33"/>
+      <c r="R43" s="33"/>
+      <c r="S43" s="33"/>
+      <c r="T43" s="33"/>
+      <c r="U43" s="33"/>
+      <c r="V43" s="33"/>
+      <c r="W43" s="34"/>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A44" s="32"/>
+      <c r="B44" s="33"/>
+      <c r="C44" s="33"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="33"/>
+      <c r="F44" s="33"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="33"/>
+      <c r="I44" s="33"/>
+      <c r="J44" s="33"/>
+      <c r="K44" s="33"/>
+      <c r="L44" s="33"/>
+      <c r="M44" s="33"/>
+      <c r="N44" s="33"/>
+      <c r="O44" s="33"/>
+      <c r="P44" s="33"/>
+      <c r="Q44" s="33"/>
+      <c r="R44" s="33"/>
+      <c r="S44" s="33"/>
+      <c r="T44" s="33"/>
+      <c r="U44" s="33"/>
+      <c r="V44" s="33"/>
+      <c r="W44" s="34"/>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A45" s="32"/>
+      <c r="B45" s="33"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="33"/>
+      <c r="H45" s="33"/>
+      <c r="I45" s="33"/>
+      <c r="J45" s="33"/>
+      <c r="K45" s="33"/>
+      <c r="L45" s="33"/>
+      <c r="M45" s="33"/>
+      <c r="N45" s="33"/>
+      <c r="O45" s="33"/>
+      <c r="P45" s="33"/>
+      <c r="Q45" s="33"/>
+      <c r="R45" s="33"/>
+      <c r="S45" s="33"/>
+      <c r="T45" s="33"/>
+      <c r="U45" s="33"/>
+      <c r="V45" s="33"/>
+      <c r="W45" s="34"/>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A46" s="32"/>
+      <c r="B46" s="33"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="33"/>
+      <c r="E46" s="33"/>
+      <c r="F46" s="33"/>
+      <c r="G46" s="33"/>
+      <c r="H46" s="33"/>
+      <c r="I46" s="33"/>
+      <c r="J46" s="33"/>
+      <c r="K46" s="33"/>
+      <c r="L46" s="33"/>
+      <c r="M46" s="33"/>
+      <c r="N46" s="33"/>
+      <c r="O46" s="33"/>
+      <c r="P46" s="33"/>
+      <c r="Q46" s="33"/>
+      <c r="R46" s="33"/>
+      <c r="S46" s="33"/>
+      <c r="T46" s="33"/>
+      <c r="U46" s="33"/>
+      <c r="V46" s="33"/>
+      <c r="W46" s="34"/>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A47" s="32"/>
+      <c r="B47" s="33"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="33"/>
+      <c r="J47" s="33"/>
+      <c r="K47" s="33"/>
+      <c r="L47" s="33"/>
+      <c r="M47" s="33"/>
+      <c r="N47" s="33"/>
+      <c r="O47" s="33"/>
+      <c r="P47" s="33"/>
+      <c r="Q47" s="33"/>
+      <c r="R47" s="33"/>
+      <c r="S47" s="33"/>
+      <c r="T47" s="33"/>
+      <c r="U47" s="33"/>
+      <c r="V47" s="33"/>
+      <c r="W47" s="34"/>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A48" s="32"/>
+      <c r="B48" s="33"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="33"/>
+      <c r="E48" s="33"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="33"/>
+      <c r="H48" s="33"/>
+      <c r="I48" s="33"/>
+      <c r="J48" s="33"/>
+      <c r="K48" s="33"/>
+      <c r="L48" s="33"/>
+      <c r="M48" s="33"/>
+      <c r="N48" s="33"/>
+      <c r="O48" s="33"/>
+      <c r="P48" s="33"/>
+      <c r="Q48" s="33"/>
+      <c r="R48" s="33"/>
+      <c r="S48" s="33"/>
+      <c r="T48" s="33"/>
+      <c r="U48" s="33"/>
+      <c r="V48" s="33"/>
+      <c r="W48" s="34"/>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A49" s="32"/>
+      <c r="B49" s="33"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="33"/>
+      <c r="F49" s="33"/>
+      <c r="G49" s="33"/>
+      <c r="H49" s="33"/>
+      <c r="I49" s="33"/>
+      <c r="J49" s="33"/>
+      <c r="K49" s="33"/>
+      <c r="L49" s="33"/>
+      <c r="M49" s="33"/>
+      <c r="N49" s="33"/>
+      <c r="O49" s="33"/>
+      <c r="P49" s="33"/>
+      <c r="Q49" s="33"/>
+      <c r="R49" s="33"/>
+      <c r="S49" s="33"/>
+      <c r="T49" s="33"/>
+      <c r="U49" s="33"/>
+      <c r="V49" s="33"/>
+      <c r="W49" s="34"/>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A50" s="32"/>
+      <c r="B50" s="33"/>
+      <c r="C50" s="33"/>
+      <c r="D50" s="33"/>
+      <c r="E50" s="33"/>
+      <c r="F50" s="33"/>
+      <c r="G50" s="33"/>
+      <c r="H50" s="33"/>
+      <c r="I50" s="33"/>
+      <c r="J50" s="33"/>
+      <c r="K50" s="33"/>
+      <c r="L50" s="33"/>
+      <c r="M50" s="33"/>
+      <c r="N50" s="33"/>
+      <c r="O50" s="33"/>
+      <c r="P50" s="33"/>
+      <c r="Q50" s="33"/>
+      <c r="R50" s="33"/>
+      <c r="S50" s="33"/>
+      <c r="T50" s="33"/>
+      <c r="U50" s="33"/>
+      <c r="V50" s="33"/>
+      <c r="W50" s="34"/>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A51" s="32"/>
+      <c r="B51" s="33"/>
+      <c r="C51" s="33"/>
+      <c r="D51" s="33"/>
+      <c r="E51" s="33"/>
+      <c r="F51" s="33"/>
+      <c r="G51" s="33"/>
+      <c r="H51" s="33"/>
+      <c r="I51" s="33"/>
+      <c r="J51" s="33"/>
+      <c r="K51" s="33"/>
+      <c r="L51" s="33"/>
+      <c r="M51" s="33"/>
+      <c r="N51" s="33"/>
+      <c r="O51" s="33"/>
+      <c r="P51" s="33"/>
+      <c r="Q51" s="33"/>
+      <c r="R51" s="33"/>
+      <c r="S51" s="33"/>
+      <c r="T51" s="33"/>
+      <c r="U51" s="33"/>
+      <c r="V51" s="33"/>
+      <c r="W51" s="34"/>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A52" s="32"/>
+      <c r="B52" s="33"/>
+      <c r="C52" s="33"/>
+      <c r="D52" s="33"/>
+      <c r="E52" s="33"/>
+      <c r="F52" s="33"/>
+      <c r="G52" s="33"/>
+      <c r="H52" s="33"/>
+      <c r="I52" s="33"/>
+      <c r="J52" s="33"/>
+      <c r="K52" s="33"/>
+      <c r="L52" s="33"/>
+      <c r="M52" s="33"/>
+      <c r="N52" s="33"/>
+      <c r="O52" s="33"/>
+      <c r="P52" s="33"/>
+      <c r="Q52" s="33"/>
+      <c r="R52" s="33"/>
+      <c r="S52" s="33"/>
+      <c r="T52" s="33"/>
+      <c r="U52" s="33"/>
+      <c r="V52" s="33"/>
+      <c r="W52" s="34"/>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A53" s="32"/>
+      <c r="B53" s="33"/>
+      <c r="C53" s="33"/>
+      <c r="D53" s="33"/>
+      <c r="E53" s="33"/>
+      <c r="F53" s="33"/>
+      <c r="G53" s="33"/>
+      <c r="H53" s="33"/>
+      <c r="I53" s="33"/>
+      <c r="J53" s="33"/>
+      <c r="K53" s="33"/>
+      <c r="L53" s="33"/>
+      <c r="M53" s="33"/>
+      <c r="N53" s="33"/>
+      <c r="O53" s="33"/>
+      <c r="P53" s="33"/>
+      <c r="Q53" s="33"/>
+      <c r="R53" s="33"/>
+      <c r="S53" s="33"/>
+      <c r="T53" s="33"/>
+      <c r="U53" s="33"/>
+      <c r="V53" s="33"/>
+      <c r="W53" s="34"/>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A54" s="32"/>
+      <c r="B54" s="33"/>
+      <c r="C54" s="33"/>
+      <c r="D54" s="33"/>
+      <c r="E54" s="33"/>
+      <c r="F54" s="33"/>
+      <c r="G54" s="33"/>
+      <c r="H54" s="33"/>
+      <c r="I54" s="33"/>
+      <c r="J54" s="33"/>
+      <c r="K54" s="33"/>
+      <c r="L54" s="33"/>
+      <c r="M54" s="33"/>
+      <c r="N54" s="33"/>
+      <c r="O54" s="33"/>
+      <c r="P54" s="33"/>
+      <c r="Q54" s="33"/>
+      <c r="R54" s="33"/>
+      <c r="S54" s="33"/>
+      <c r="T54" s="33"/>
+      <c r="U54" s="33"/>
+      <c r="V54" s="33"/>
+      <c r="W54" s="34"/>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A55" s="32"/>
+      <c r="B55" s="33"/>
+      <c r="C55" s="33"/>
+      <c r="D55" s="33"/>
+      <c r="E55" s="33"/>
+      <c r="F55" s="33"/>
+      <c r="G55" s="33"/>
+      <c r="H55" s="33"/>
+      <c r="I55" s="33"/>
+      <c r="J55" s="33"/>
+      <c r="K55" s="33"/>
+      <c r="L55" s="33"/>
+      <c r="M55" s="33"/>
+      <c r="N55" s="33"/>
+      <c r="O55" s="33"/>
+      <c r="P55" s="33"/>
+      <c r="Q55" s="33"/>
+      <c r="R55" s="33"/>
+      <c r="S55" s="33"/>
+      <c r="T55" s="33"/>
+      <c r="U55" s="33"/>
+      <c r="V55" s="33"/>
+      <c r="W55" s="34"/>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A56" s="32"/>
+      <c r="B56" s="33"/>
+      <c r="C56" s="33"/>
+      <c r="D56" s="33"/>
+      <c r="E56" s="33"/>
+      <c r="F56" s="33"/>
+      <c r="G56" s="33"/>
+      <c r="H56" s="33"/>
+      <c r="I56" s="33"/>
+      <c r="J56" s="33"/>
+      <c r="K56" s="33"/>
+      <c r="L56" s="33"/>
+      <c r="M56" s="33"/>
+      <c r="N56" s="33"/>
+      <c r="O56" s="33"/>
+      <c r="P56" s="33"/>
+      <c r="Q56" s="33"/>
+      <c r="R56" s="33"/>
+      <c r="S56" s="33"/>
+      <c r="T56" s="33"/>
+      <c r="U56" s="33"/>
+      <c r="V56" s="33"/>
+      <c r="W56" s="34"/>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A57" s="32"/>
+      <c r="B57" s="33"/>
+      <c r="C57" s="33"/>
+      <c r="D57" s="33"/>
+      <c r="E57" s="33"/>
+      <c r="F57" s="33"/>
+      <c r="G57" s="33"/>
+      <c r="H57" s="33"/>
+      <c r="I57" s="33"/>
+      <c r="J57" s="33"/>
+      <c r="K57" s="33"/>
+      <c r="L57" s="33"/>
+      <c r="M57" s="33"/>
+      <c r="N57" s="33"/>
+      <c r="O57" s="33"/>
+      <c r="P57" s="33"/>
+      <c r="Q57" s="33"/>
+      <c r="R57" s="33"/>
+      <c r="S57" s="33"/>
+      <c r="T57" s="33"/>
+      <c r="U57" s="33"/>
+      <c r="V57" s="33"/>
+      <c r="W57" s="34"/>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A58" s="32"/>
+      <c r="B58" s="33"/>
+      <c r="C58" s="33"/>
+      <c r="D58" s="33"/>
+      <c r="E58" s="33"/>
+      <c r="F58" s="33"/>
+      <c r="G58" s="33"/>
+      <c r="H58" s="33"/>
+      <c r="I58" s="33"/>
+      <c r="J58" s="33"/>
+      <c r="K58" s="33"/>
+      <c r="L58" s="33"/>
+      <c r="M58" s="33"/>
+      <c r="N58" s="33"/>
+      <c r="O58" s="33"/>
+      <c r="P58" s="33"/>
+      <c r="Q58" s="33"/>
+      <c r="R58" s="33"/>
+      <c r="S58" s="33"/>
+      <c r="T58" s="33"/>
+      <c r="U58" s="33"/>
+      <c r="V58" s="33"/>
+      <c r="W58" s="34"/>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A59" s="32"/>
+      <c r="B59" s="33"/>
+      <c r="C59" s="33"/>
+      <c r="D59" s="33"/>
+      <c r="E59" s="33"/>
+      <c r="F59" s="33"/>
+      <c r="G59" s="33"/>
+      <c r="H59" s="33"/>
+      <c r="I59" s="33"/>
+      <c r="J59" s="33"/>
+      <c r="K59" s="33"/>
+      <c r="L59" s="33"/>
+      <c r="M59" s="33"/>
+      <c r="N59" s="33"/>
+      <c r="O59" s="33"/>
+      <c r="P59" s="33"/>
+      <c r="Q59" s="33"/>
+      <c r="R59" s="33"/>
+      <c r="S59" s="33"/>
+      <c r="T59" s="33"/>
+      <c r="U59" s="33"/>
+      <c r="V59" s="33"/>
+      <c r="W59" s="34"/>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A60" s="32"/>
+      <c r="B60" s="33"/>
+      <c r="C60" s="33"/>
+      <c r="D60" s="33"/>
+      <c r="E60" s="33"/>
+      <c r="F60" s="33"/>
+      <c r="G60" s="33"/>
+      <c r="H60" s="33"/>
+      <c r="I60" s="33"/>
+      <c r="J60" s="33"/>
+      <c r="K60" s="33"/>
+      <c r="L60" s="33"/>
+      <c r="M60" s="33"/>
+      <c r="N60" s="33"/>
+      <c r="O60" s="33"/>
+      <c r="P60" s="33"/>
+      <c r="Q60" s="33"/>
+      <c r="R60" s="33"/>
+      <c r="S60" s="33"/>
+      <c r="T60" s="33"/>
+      <c r="U60" s="33"/>
+      <c r="V60" s="33"/>
+      <c r="W60" s="34"/>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A61" s="32"/>
+      <c r="B61" s="33"/>
+      <c r="C61" s="33"/>
+      <c r="D61" s="33"/>
+      <c r="E61" s="33"/>
+      <c r="F61" s="33"/>
+      <c r="G61" s="33"/>
+      <c r="H61" s="33"/>
+      <c r="I61" s="33"/>
+      <c r="J61" s="33"/>
+      <c r="K61" s="33"/>
+      <c r="L61" s="33"/>
+      <c r="M61" s="33"/>
+      <c r="N61" s="33"/>
+      <c r="O61" s="33"/>
+      <c r="P61" s="33"/>
+      <c r="Q61" s="33"/>
+      <c r="R61" s="33"/>
+      <c r="S61" s="33"/>
+      <c r="T61" s="33"/>
+      <c r="U61" s="33"/>
+      <c r="V61" s="33"/>
+      <c r="W61" s="34"/>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A62" s="32"/>
+      <c r="B62" s="33"/>
+      <c r="C62" s="33"/>
+      <c r="D62" s="33"/>
+      <c r="E62" s="33"/>
+      <c r="F62" s="33"/>
+      <c r="G62" s="33"/>
+      <c r="H62" s="33"/>
+      <c r="I62" s="33"/>
+      <c r="J62" s="33"/>
+      <c r="K62" s="33"/>
+      <c r="L62" s="33"/>
+      <c r="M62" s="33"/>
+      <c r="N62" s="33"/>
+      <c r="O62" s="33"/>
+      <c r="P62" s="33"/>
+      <c r="Q62" s="33"/>
+      <c r="R62" s="33"/>
+      <c r="S62" s="33"/>
+      <c r="T62" s="33"/>
+      <c r="U62" s="33"/>
+      <c r="V62" s="33"/>
+      <c r="W62" s="34"/>
+    </row>
+    <row r="63" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A63" s="35"/>
+      <c r="B63" s="36"/>
+      <c r="C63" s="36"/>
+      <c r="D63" s="36"/>
+      <c r="E63" s="36"/>
+      <c r="F63" s="36"/>
+      <c r="G63" s="36"/>
+      <c r="H63" s="36"/>
+      <c r="I63" s="36"/>
+      <c r="J63" s="36"/>
+      <c r="K63" s="36"/>
+      <c r="L63" s="36"/>
+      <c r="M63" s="36"/>
+      <c r="N63" s="36"/>
+      <c r="O63" s="36"/>
+      <c r="P63" s="36"/>
+      <c r="Q63" s="36"/>
+      <c r="R63" s="36"/>
+      <c r="S63" s="36"/>
+      <c r="T63" s="36"/>
+      <c r="U63" s="36"/>
+      <c r="V63" s="36"/>
+      <c r="W63" s="37"/>
+    </row>
+    <row r="64" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A64" s="38"/>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A65" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="B65" s="40"/>
+      <c r="C65" s="40"/>
+      <c r="D65" s="40"/>
+      <c r="E65" s="40"/>
+      <c r="F65" s="40"/>
+      <c r="G65" s="40"/>
+      <c r="H65" s="40"/>
+      <c r="I65" s="40"/>
+      <c r="J65" s="40"/>
+      <c r="K65" s="40"/>
+      <c r="L65" s="40"/>
+      <c r="M65" s="40"/>
+      <c r="N65" s="40"/>
+      <c r="O65" s="40"/>
+      <c r="P65" s="40"/>
+      <c r="Q65" s="40"/>
+      <c r="R65" s="40"/>
+      <c r="S65" s="40"/>
+      <c r="T65" s="40"/>
+      <c r="U65" s="40"/>
+      <c r="V65" s="40"/>
+      <c r="W65" s="41"/>
+    </row>
+    <row r="66" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A66" s="42"/>
+      <c r="B66" s="43"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="43"/>
+      <c r="I66" s="43"/>
+      <c r="J66" s="43"/>
+      <c r="K66" s="43"/>
+      <c r="L66" s="43"/>
+      <c r="M66" s="43"/>
+      <c r="N66" s="43"/>
+      <c r="O66" s="43"/>
+      <c r="P66" s="43"/>
+      <c r="Q66" s="43"/>
+      <c r="R66" s="43"/>
+      <c r="S66" s="43"/>
+      <c r="T66" s="43"/>
+      <c r="U66" s="43"/>
+      <c r="V66" s="43"/>
+      <c r="W66" s="44"/>
+    </row>
+    <row r="67" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A67" s="45" t="s">
         <v>110</v>
       </c>
-      <c r="M17" s="26"/>
-      <c r="N17" s="26"/>
-      <c r="O17" s="26"/>
-      <c r="P17" s="26"/>
-      <c r="Q17" s="26"/>
-      <c r="R17" s="26"/>
-      <c r="S17" s="26"/>
-      <c r="T17" s="26"/>
-      <c r="U17" s="26"/>
-      <c r="V17" s="26"/>
-      <c r="W17" s="27"/>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A18" s="28"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="31"/>
-      <c r="M18" s="32"/>
-      <c r="N18" s="32"/>
-      <c r="O18" s="32"/>
-      <c r="P18" s="32"/>
-      <c r="Q18" s="32"/>
-      <c r="R18" s="32"/>
-      <c r="S18" s="32"/>
-      <c r="T18" s="32"/>
-      <c r="U18" s="32"/>
-      <c r="V18" s="32"/>
-      <c r="W18" s="33"/>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A19" s="28"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
-      <c r="J19" s="29"/>
-      <c r="K19" s="30"/>
-      <c r="L19" s="31"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="32"/>
-      <c r="O19" s="32"/>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="32"/>
-      <c r="S19" s="32"/>
-      <c r="T19" s="32"/>
-      <c r="U19" s="32"/>
-      <c r="V19" s="32"/>
-      <c r="W19" s="33"/>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A20" s="28"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="30"/>
-      <c r="L20" s="31"/>
-      <c r="M20" s="32"/>
-      <c r="N20" s="32"/>
-      <c r="O20" s="32"/>
-      <c r="P20" s="32"/>
-      <c r="Q20" s="32"/>
-      <c r="R20" s="32"/>
-      <c r="S20" s="32"/>
-      <c r="T20" s="32"/>
-      <c r="U20" s="32"/>
-      <c r="V20" s="32"/>
-      <c r="W20" s="33"/>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A21" s="28"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="29"/>
-      <c r="H21" s="29"/>
-      <c r="I21" s="29"/>
-      <c r="J21" s="29"/>
-      <c r="K21" s="30"/>
-      <c r="L21" s="31"/>
-      <c r="M21" s="32"/>
-      <c r="N21" s="32"/>
-      <c r="O21" s="32"/>
-      <c r="P21" s="32"/>
-      <c r="Q21" s="32"/>
-      <c r="R21" s="32"/>
-      <c r="S21" s="32"/>
-      <c r="T21" s="32"/>
-      <c r="U21" s="32"/>
-      <c r="V21" s="32"/>
-      <c r="W21" s="33"/>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="29"/>
-      <c r="I22" s="29"/>
-      <c r="J22" s="29"/>
-      <c r="K22" s="30"/>
-      <c r="L22" s="31"/>
-      <c r="M22" s="32"/>
-      <c r="N22" s="32"/>
-      <c r="O22" s="32"/>
-      <c r="P22" s="32"/>
-      <c r="Q22" s="32"/>
-      <c r="R22" s="32"/>
-      <c r="S22" s="32"/>
-      <c r="T22" s="32"/>
-      <c r="U22" s="32"/>
-      <c r="V22" s="32"/>
-      <c r="W22" s="33"/>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A23" s="28"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="30"/>
-      <c r="L23" s="31"/>
-      <c r="M23" s="32"/>
-      <c r="N23" s="32"/>
-      <c r="O23" s="32"/>
-      <c r="P23" s="32"/>
-      <c r="Q23" s="32"/>
-      <c r="R23" s="32"/>
-      <c r="S23" s="32"/>
-      <c r="T23" s="32"/>
-      <c r="U23" s="32"/>
-      <c r="V23" s="32"/>
-      <c r="W23" s="33"/>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A24" s="28"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="29"/>
-      <c r="G24" s="29"/>
-      <c r="H24" s="29"/>
-      <c r="I24" s="29"/>
-      <c r="J24" s="29"/>
-      <c r="K24" s="30"/>
-      <c r="L24" s="31"/>
-      <c r="M24" s="32"/>
-      <c r="N24" s="32"/>
-      <c r="O24" s="32"/>
-      <c r="P24" s="32"/>
-      <c r="Q24" s="32"/>
-      <c r="R24" s="32"/>
-      <c r="S24" s="32"/>
-      <c r="T24" s="32"/>
-      <c r="U24" s="32"/>
-      <c r="V24" s="32"/>
-      <c r="W24" s="33"/>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A25" s="28"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="29"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="29"/>
-      <c r="K25" s="30"/>
-      <c r="L25" s="31"/>
-      <c r="M25" s="32"/>
-      <c r="N25" s="32"/>
-      <c r="O25" s="32"/>
-      <c r="P25" s="32"/>
-      <c r="Q25" s="32"/>
-      <c r="R25" s="32"/>
-      <c r="S25" s="32"/>
-      <c r="T25" s="32"/>
-      <c r="U25" s="32"/>
-      <c r="V25" s="32"/>
-      <c r="W25" s="33"/>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A26" s="28"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="29"/>
-      <c r="K26" s="30"/>
-      <c r="L26" s="31"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="32"/>
-      <c r="O26" s="32"/>
-      <c r="P26" s="32"/>
-      <c r="Q26" s="32"/>
-      <c r="R26" s="32"/>
-      <c r="S26" s="32"/>
-      <c r="T26" s="32"/>
-      <c r="U26" s="32"/>
-      <c r="V26" s="32"/>
-      <c r="W26" s="33"/>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A27" s="28"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="29"/>
-      <c r="K27" s="30"/>
-      <c r="L27" s="31"/>
-      <c r="M27" s="32"/>
-      <c r="N27" s="32"/>
-      <c r="O27" s="32"/>
-      <c r="P27" s="32"/>
-      <c r="Q27" s="32"/>
-      <c r="R27" s="32"/>
-      <c r="S27" s="32"/>
-      <c r="T27" s="32"/>
-      <c r="U27" s="32"/>
-      <c r="V27" s="32"/>
-      <c r="W27" s="33"/>
-    </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A28" s="28"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
-      <c r="H28" s="29"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="30"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="32"/>
-      <c r="N28" s="32"/>
-      <c r="O28" s="32"/>
-      <c r="P28" s="32"/>
-      <c r="Q28" s="32"/>
-      <c r="R28" s="32"/>
-      <c r="S28" s="32"/>
-      <c r="T28" s="32"/>
-      <c r="U28" s="32"/>
-      <c r="V28" s="32"/>
-      <c r="W28" s="33"/>
-    </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A29" s="28"/>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29"/>
-      <c r="H29" s="29"/>
-      <c r="I29" s="29"/>
-      <c r="J29" s="29"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="31"/>
-      <c r="M29" s="32"/>
-      <c r="N29" s="32"/>
-      <c r="O29" s="32"/>
-      <c r="P29" s="32"/>
-      <c r="Q29" s="32"/>
-      <c r="R29" s="32"/>
-      <c r="S29" s="32"/>
-      <c r="T29" s="32"/>
-      <c r="U29" s="32"/>
-      <c r="V29" s="32"/>
-      <c r="W29" s="33"/>
-    </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A30" s="28"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
-      <c r="G30" s="29"/>
-      <c r="H30" s="29"/>
-      <c r="I30" s="29"/>
-      <c r="J30" s="29"/>
-      <c r="K30" s="30"/>
-      <c r="L30" s="31"/>
-      <c r="M30" s="32"/>
-      <c r="N30" s="32"/>
-      <c r="O30" s="32"/>
-      <c r="P30" s="32"/>
-      <c r="Q30" s="32"/>
-      <c r="R30" s="32"/>
-      <c r="S30" s="32"/>
-      <c r="T30" s="32"/>
-      <c r="U30" s="32"/>
-      <c r="V30" s="32"/>
-      <c r="W30" s="33"/>
-    </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A31" s="28"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
-      <c r="G31" s="29"/>
-      <c r="H31" s="29"/>
-      <c r="I31" s="29"/>
-      <c r="J31" s="29"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="31"/>
-      <c r="M31" s="32"/>
-      <c r="N31" s="32"/>
-      <c r="O31" s="32"/>
-      <c r="P31" s="32"/>
-      <c r="Q31" s="32"/>
-      <c r="R31" s="32"/>
-      <c r="S31" s="32"/>
-      <c r="T31" s="32"/>
-      <c r="U31" s="32"/>
-      <c r="V31" s="32"/>
-      <c r="W31" s="33"/>
-    </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A32" s="28"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="29"/>
-      <c r="J32" s="29"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="31"/>
-      <c r="M32" s="32"/>
-      <c r="N32" s="32"/>
-      <c r="O32" s="32"/>
-      <c r="P32" s="32"/>
-      <c r="Q32" s="32"/>
-      <c r="R32" s="32"/>
-      <c r="S32" s="32"/>
-      <c r="T32" s="32"/>
-      <c r="U32" s="32"/>
-      <c r="V32" s="32"/>
-      <c r="W32" s="33"/>
-    </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A33" s="28"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="29"/>
-      <c r="H33" s="29"/>
-      <c r="I33" s="29"/>
-      <c r="J33" s="29"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="31"/>
-      <c r="M33" s="32"/>
-      <c r="N33" s="32"/>
-      <c r="O33" s="32"/>
-      <c r="P33" s="32"/>
-      <c r="Q33" s="32"/>
-      <c r="R33" s="32"/>
-      <c r="S33" s="32"/>
-      <c r="T33" s="32"/>
-      <c r="U33" s="32"/>
-      <c r="V33" s="32"/>
-      <c r="W33" s="33"/>
-    </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A34" s="28"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="29"/>
-      <c r="F34" s="29"/>
-      <c r="G34" s="29"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="29"/>
-      <c r="J34" s="29"/>
-      <c r="K34" s="30"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="32"/>
-      <c r="N34" s="32"/>
-      <c r="O34" s="32"/>
-      <c r="P34" s="32"/>
-      <c r="Q34" s="32"/>
-      <c r="R34" s="32"/>
-      <c r="S34" s="32"/>
-      <c r="T34" s="32"/>
-      <c r="U34" s="32"/>
-      <c r="V34" s="32"/>
-      <c r="W34" s="33"/>
-    </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A35" s="28"/>
-      <c r="B35" s="29"/>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="29"/>
-      <c r="F35" s="29"/>
-      <c r="G35" s="29"/>
-      <c r="H35" s="29"/>
-      <c r="I35" s="29"/>
-      <c r="J35" s="29"/>
-      <c r="K35" s="30"/>
-      <c r="L35" s="31"/>
-      <c r="M35" s="32"/>
-      <c r="N35" s="32"/>
-      <c r="O35" s="32"/>
-      <c r="P35" s="32"/>
-      <c r="Q35" s="32"/>
-      <c r="R35" s="32"/>
-      <c r="S35" s="32"/>
-      <c r="T35" s="32"/>
-      <c r="U35" s="32"/>
-      <c r="V35" s="32"/>
-      <c r="W35" s="33"/>
-    </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A36" s="28"/>
-      <c r="B36" s="29"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="29"/>
-      <c r="F36" s="29"/>
-      <c r="G36" s="29"/>
-      <c r="H36" s="29"/>
-      <c r="I36" s="29"/>
-      <c r="J36" s="29"/>
-      <c r="K36" s="30"/>
-      <c r="L36" s="31"/>
-      <c r="M36" s="32"/>
-      <c r="N36" s="32"/>
-      <c r="O36" s="32"/>
-      <c r="P36" s="32"/>
-      <c r="Q36" s="32"/>
-      <c r="R36" s="32"/>
-      <c r="S36" s="32"/>
-      <c r="T36" s="32"/>
-      <c r="U36" s="32"/>
-      <c r="V36" s="32"/>
-      <c r="W36" s="33"/>
-    </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A37" s="28"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="29"/>
-      <c r="H37" s="29"/>
-      <c r="I37" s="29"/>
-      <c r="J37" s="29"/>
-      <c r="K37" s="30"/>
-      <c r="L37" s="31"/>
-      <c r="M37" s="32"/>
-      <c r="N37" s="32"/>
-      <c r="O37" s="32"/>
-      <c r="P37" s="32"/>
-      <c r="Q37" s="32"/>
-      <c r="R37" s="32"/>
-      <c r="S37" s="32"/>
-      <c r="T37" s="32"/>
-      <c r="U37" s="32"/>
-      <c r="V37" s="32"/>
-      <c r="W37" s="33"/>
-    </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A38" s="28"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="29"/>
-      <c r="J38" s="29"/>
-      <c r="K38" s="30"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="32"/>
-      <c r="N38" s="32"/>
-      <c r="O38" s="32"/>
-      <c r="P38" s="32"/>
-      <c r="Q38" s="32"/>
-      <c r="R38" s="32"/>
-      <c r="S38" s="32"/>
-      <c r="T38" s="32"/>
-      <c r="U38" s="32"/>
-      <c r="V38" s="32"/>
-      <c r="W38" s="33"/>
-    </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A39" s="28"/>
-      <c r="B39" s="29"/>
-      <c r="C39" s="29"/>
-      <c r="D39" s="29"/>
-      <c r="E39" s="29"/>
-      <c r="F39" s="29"/>
-      <c r="G39" s="29"/>
-      <c r="H39" s="29"/>
-      <c r="I39" s="29"/>
-      <c r="J39" s="29"/>
-      <c r="K39" s="30"/>
-      <c r="L39" s="31"/>
-      <c r="M39" s="32"/>
-      <c r="N39" s="32"/>
-      <c r="O39" s="32"/>
-      <c r="P39" s="32"/>
-      <c r="Q39" s="32"/>
-      <c r="R39" s="32"/>
-      <c r="S39" s="32"/>
-      <c r="T39" s="32"/>
-      <c r="U39" s="32"/>
-      <c r="V39" s="32"/>
-      <c r="W39" s="33"/>
-    </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A40" s="28"/>
-      <c r="B40" s="29"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="29"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="30"/>
-      <c r="L40" s="31"/>
-      <c r="M40" s="32"/>
-      <c r="N40" s="32"/>
-      <c r="O40" s="32"/>
-      <c r="P40" s="32"/>
-      <c r="Q40" s="32"/>
-      <c r="R40" s="32"/>
-      <c r="S40" s="32"/>
-      <c r="T40" s="32"/>
-      <c r="U40" s="32"/>
-      <c r="V40" s="32"/>
-      <c r="W40" s="33"/>
-    </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A41" s="28"/>
-      <c r="B41" s="29"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="29"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="29"/>
-      <c r="H41" s="29"/>
-      <c r="I41" s="29"/>
-      <c r="J41" s="29"/>
-      <c r="K41" s="30"/>
-      <c r="L41" s="31"/>
-      <c r="M41" s="32"/>
-      <c r="N41" s="32"/>
-      <c r="O41" s="32"/>
-      <c r="P41" s="32"/>
-      <c r="Q41" s="32"/>
-      <c r="R41" s="32"/>
-      <c r="S41" s="32"/>
-      <c r="T41" s="32"/>
-      <c r="U41" s="32"/>
-      <c r="V41" s="32"/>
-      <c r="W41" s="33"/>
-    </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="28"/>
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
-      <c r="H42" s="29"/>
-      <c r="I42" s="29"/>
-      <c r="J42" s="29"/>
-      <c r="K42" s="30"/>
-      <c r="L42" s="31"/>
-      <c r="M42" s="32"/>
-      <c r="N42" s="32"/>
-      <c r="O42" s="32"/>
-      <c r="P42" s="32"/>
-      <c r="Q42" s="32"/>
-      <c r="R42" s="32"/>
-      <c r="S42" s="32"/>
-      <c r="T42" s="32"/>
-      <c r="U42" s="32"/>
-      <c r="V42" s="32"/>
-      <c r="W42" s="33"/>
-    </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A43" s="28"/>
-      <c r="B43" s="29"/>
-      <c r="C43" s="29"/>
-      <c r="D43" s="29"/>
-      <c r="E43" s="29"/>
-      <c r="F43" s="29"/>
-      <c r="G43" s="29"/>
-      <c r="H43" s="29"/>
-      <c r="I43" s="29"/>
-      <c r="J43" s="29"/>
-      <c r="K43" s="30"/>
-      <c r="L43" s="31"/>
-      <c r="M43" s="32"/>
-      <c r="N43" s="32"/>
-      <c r="O43" s="32"/>
-      <c r="P43" s="32"/>
-      <c r="Q43" s="32"/>
-      <c r="R43" s="32"/>
-      <c r="S43" s="32"/>
-      <c r="T43" s="32"/>
-      <c r="U43" s="32"/>
-      <c r="V43" s="32"/>
-      <c r="W43" s="33"/>
-    </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A44" s="28"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="29"/>
-      <c r="E44" s="29"/>
-      <c r="F44" s="29"/>
-      <c r="G44" s="29"/>
-      <c r="H44" s="29"/>
-      <c r="I44" s="29"/>
-      <c r="J44" s="29"/>
-      <c r="K44" s="30"/>
-      <c r="L44" s="31"/>
-      <c r="M44" s="32"/>
-      <c r="N44" s="32"/>
-      <c r="O44" s="32"/>
-      <c r="P44" s="32"/>
-      <c r="Q44" s="32"/>
-      <c r="R44" s="32"/>
-      <c r="S44" s="32"/>
-      <c r="T44" s="32"/>
-      <c r="U44" s="32"/>
-      <c r="V44" s="32"/>
-      <c r="W44" s="33"/>
-    </row>
-    <row r="45" spans="1:23" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="28"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="29"/>
-      <c r="D45" s="29"/>
-      <c r="E45" s="29"/>
-      <c r="F45" s="29"/>
-      <c r="G45" s="29"/>
-      <c r="H45" s="29"/>
-      <c r="I45" s="29"/>
-      <c r="J45" s="29"/>
-      <c r="K45" s="30"/>
-      <c r="L45" s="31"/>
-      <c r="M45" s="32"/>
-      <c r="N45" s="32"/>
-      <c r="O45" s="32"/>
-      <c r="P45" s="32"/>
-      <c r="Q45" s="32"/>
-      <c r="R45" s="32"/>
-      <c r="S45" s="32"/>
-      <c r="T45" s="32"/>
-      <c r="U45" s="32"/>
-      <c r="V45" s="32"/>
-      <c r="W45" s="33"/>
-    </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A46" s="28"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="29"/>
-      <c r="E46" s="29"/>
-      <c r="F46" s="29"/>
-      <c r="G46" s="29"/>
-      <c r="H46" s="29"/>
-      <c r="I46" s="29"/>
-      <c r="J46" s="29"/>
-      <c r="K46" s="30"/>
-      <c r="L46" s="31"/>
-      <c r="M46" s="32"/>
-      <c r="N46" s="32"/>
-      <c r="O46" s="32"/>
-      <c r="P46" s="32"/>
-      <c r="Q46" s="32"/>
-      <c r="R46" s="32"/>
-      <c r="S46" s="32"/>
-      <c r="T46" s="32"/>
-      <c r="U46" s="32"/>
-      <c r="V46" s="32"/>
-      <c r="W46" s="33"/>
-    </row>
-    <row r="47" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="34"/>
-      <c r="B47" s="35"/>
-      <c r="C47" s="35"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="35"/>
-      <c r="F47" s="35"/>
-      <c r="G47" s="35"/>
-      <c r="H47" s="35"/>
-      <c r="I47" s="35"/>
-      <c r="J47" s="35"/>
-      <c r="K47" s="36"/>
-      <c r="L47" s="37"/>
-      <c r="M47" s="38"/>
-      <c r="N47" s="38"/>
-      <c r="O47" s="38"/>
-      <c r="P47" s="38"/>
-      <c r="Q47" s="38"/>
-      <c r="R47" s="38"/>
-      <c r="S47" s="38"/>
-      <c r="T47" s="38"/>
-      <c r="U47" s="38"/>
-      <c r="V47" s="38"/>
-      <c r="W47" s="39"/>
-    </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A48" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="B48" s="41"/>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="41"/>
-      <c r="I48" s="41"/>
-      <c r="J48" s="41"/>
-      <c r="K48" s="41"/>
-      <c r="L48" s="41"/>
-      <c r="M48" s="41"/>
-      <c r="N48" s="41"/>
-      <c r="O48" s="41"/>
-      <c r="P48" s="41"/>
-      <c r="Q48" s="41"/>
-      <c r="R48" s="41"/>
-      <c r="S48" s="41"/>
-      <c r="T48" s="41"/>
-      <c r="U48" s="41"/>
-      <c r="V48" s="41"/>
-      <c r="W48" s="42"/>
-    </row>
-    <row r="49" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="43"/>
-      <c r="B49" s="44"/>
-      <c r="C49" s="44"/>
-      <c r="D49" s="44"/>
-      <c r="E49" s="44"/>
-      <c r="F49" s="44"/>
-      <c r="G49" s="44"/>
-      <c r="H49" s="44"/>
-      <c r="I49" s="44"/>
-      <c r="J49" s="44"/>
-      <c r="K49" s="44"/>
-      <c r="L49" s="44"/>
-      <c r="M49" s="44"/>
-      <c r="N49" s="44"/>
-      <c r="O49" s="44"/>
-      <c r="P49" s="44"/>
-      <c r="Q49" s="44"/>
-      <c r="R49" s="44"/>
-      <c r="S49" s="44"/>
-      <c r="T49" s="44"/>
-      <c r="U49" s="44"/>
-      <c r="V49" s="44"/>
-      <c r="W49" s="45"/>
-    </row>
-    <row r="50" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="46" t="s">
-        <v>112</v>
-      </c>
-      <c r="B50" s="47"/>
-      <c r="C50" s="47"/>
-      <c r="D50" s="47"/>
-      <c r="E50" s="47"/>
-      <c r="F50" s="47"/>
-      <c r="G50" s="47"/>
-      <c r="H50" s="47"/>
-      <c r="I50" s="47"/>
-      <c r="J50" s="47"/>
-      <c r="K50" s="47"/>
-      <c r="L50" s="47"/>
-      <c r="M50" s="47"/>
-      <c r="N50" s="47"/>
-      <c r="O50" s="47"/>
-      <c r="P50" s="47"/>
-      <c r="Q50" s="47"/>
-      <c r="R50" s="47"/>
-      <c r="S50" s="47"/>
-      <c r="T50" s="47"/>
-      <c r="U50" s="47"/>
-      <c r="V50" s="47"/>
-      <c r="W50" s="48"/>
-    </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="S51" s="49" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A59" s="50"/>
-    </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A60" s="51"/>
-    </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A61" s="51"/>
-    </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A62" s="51"/>
-    </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A63" s="51"/>
-    </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A64" s="51"/>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" s="51"/>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" s="51"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" s="51"/>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" s="51"/>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" s="51"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" s="51"/>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" s="51"/>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" s="51"/>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" s="51"/>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" s="51"/>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" s="51"/>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" s="51"/>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" s="51"/>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" s="51"/>
+      <c r="B67" s="46"/>
+      <c r="C67" s="46"/>
+      <c r="D67" s="46"/>
+      <c r="E67" s="46"/>
+      <c r="F67" s="46"/>
+      <c r="G67" s="46"/>
+      <c r="H67" s="46"/>
+      <c r="I67" s="46"/>
+      <c r="J67" s="46"/>
+      <c r="K67" s="46"/>
+      <c r="L67" s="46"/>
+      <c r="M67" s="46"/>
+      <c r="N67" s="46"/>
+      <c r="O67" s="46"/>
+      <c r="P67" s="46"/>
+      <c r="Q67" s="46"/>
+      <c r="R67" s="46"/>
+      <c r="S67" s="46"/>
+      <c r="T67" s="46"/>
+      <c r="U67" s="46"/>
+      <c r="V67" s="46"/>
+      <c r="W67" s="47"/>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A68" s="38"/>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A69" s="38"/>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A70" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A48:W49"/>
-    <mergeCell ref="A50:W50"/>
+    <mergeCell ref="A65:W66"/>
+    <mergeCell ref="A67:W67"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A13:W14"/>
-    <mergeCell ref="A16:W16"/>
-    <mergeCell ref="A17:K47"/>
-    <mergeCell ref="L17:W47"/>
+    <mergeCell ref="A4:W4"/>
+    <mergeCell ref="A6:W7"/>
+    <mergeCell ref="A9:W9"/>
+    <mergeCell ref="A10:W63"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="130" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -2389,7 +3549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>3</v>
       </c>
@@ -2400,7 +3560,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="13"/>
       <c r="B3" s="3" t="s">
         <v>6</v>
@@ -2409,7 +3569,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="13"/>
       <c r="B4" s="3" t="s">
         <v>8</v>
@@ -2418,7 +3578,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="13"/>
       <c r="B5" s="3" t="s">
         <v>10</v>
@@ -2427,7 +3587,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="13"/>
       <c r="B6" s="3" t="s">
         <v>12</v>
@@ -2436,7 +3596,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="13"/>
       <c r="B7" s="3" t="s">
         <v>14</v>
@@ -2445,7 +3605,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="13"/>
       <c r="B8" s="3" t="s">
         <v>16</v>
@@ -2454,7 +3614,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="13"/>
       <c r="B9" s="3" t="s">
         <v>18</v>
@@ -2463,7 +3623,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="13"/>
       <c r="B10" s="3" t="s">
         <v>20</v>
@@ -2472,7 +3632,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="13"/>
       <c r="B11" s="3" t="s">
         <v>22</v>
@@ -2481,7 +3641,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="13"/>
       <c r="B12" s="3" t="s">
         <v>24</v>
@@ -2490,7 +3650,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="13"/>
       <c r="B13" s="3" t="s">
         <v>26</v>
@@ -2499,7 +3659,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="13"/>
       <c r="B14" s="3" t="s">
         <v>28</v>
@@ -2508,7 +3668,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="13"/>
       <c r="B15" s="3" t="s">
         <v>30</v>
@@ -2517,7 +3677,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="14"/>
       <c r="B16" s="5" t="s">
         <v>32</v>
@@ -2526,19 +3686,19 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
         <v>34</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
     </row>
-    <row r="18" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="12"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
     </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
         <v>35</v>
       </c>
@@ -2549,7 +3709,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="15"/>
       <c r="B20" s="3" t="s">
         <v>38</v>
@@ -2558,7 +3718,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="15"/>
       <c r="B21" s="3" t="s">
         <v>40</v>
@@ -2567,7 +3727,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="12"/>
       <c r="B22" s="5" t="s">
         <v>42</v>
@@ -2576,7 +3736,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="13" t="s">
         <v>44</v>
       </c>
@@ -2587,7 +3747,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="13"/>
       <c r="B24" s="3" t="s">
         <v>47</v>
@@ -2596,7 +3756,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="13"/>
       <c r="B25" s="3" t="s">
         <v>49</v>
@@ -2605,7 +3765,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="13"/>
       <c r="B26" s="3" t="s">
         <v>51</v>
@@ -2614,7 +3774,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="14"/>
       <c r="B27" s="5" t="s">
         <v>53</v>
@@ -2639,7 +3799,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AI10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
@@ -2672,7 +3832,7 @@
     <col min="35" max="35" width="9" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
@@ -2779,7 +3939,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>569</v>
       </c>
@@ -2874,7 +4034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>570</v>
       </c>
@@ -2960,7 +4120,7 @@
         <v>0.97160000000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>571</v>
       </c>
@@ -3055,7 +4215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>572</v>
       </c>
@@ -3150,7 +4310,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>573</v>
       </c>
@@ -3245,7 +4405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>574</v>
       </c>
@@ -3340,7 +4500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>575</v>
       </c>
@@ -3435,7 +4595,7 @@
         <v>0.99160000000000004</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>576</v>
       </c>
@@ -3530,7 +4690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>592</v>
       </c>
@@ -3619,7 +4779,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
@@ -3641,7 +4801,7 @@
     <col min="24" max="24" width="9" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
@@ -3715,7 +4875,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>569</v>
       </c>
@@ -3780,7 +4940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>570</v>
       </c>
@@ -3836,7 +4996,7 @@
         <v>0.97160000000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>571</v>
       </c>
@@ -3901,7 +5061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>572</v>
       </c>
@@ -3966,7 +5126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>573</v>
       </c>
@@ -4031,7 +5191,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>574</v>
       </c>
@@ -4096,7 +5256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>575</v>
       </c>
@@ -4161,7 +5321,7 @@
         <v>0.99160000000000004</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>576</v>
       </c>
@@ -4226,7 +5386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>592</v>
       </c>

</xml_diff>